<commit_message>
tambah fitur export excel menu verifikasi dokumen
</commit_message>
<xml_diff>
--- a/application/assets/excel/rekap_kontrak_pengadaan.xlsx
+++ b/application/assets/excel/rekap_kontrak_pengadaan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\noval\application\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF486D10-4FE3-4F1B-855C-AC09AD7C033B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E31A6ADF-0460-43AE-A0CE-7A7CA5FEF53E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E7A15CC7-3E23-4118-92B5-661F9C474EDE}"/>
   </bookViews>
@@ -57,13 +57,13 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Laporan Kontrak Pengadaan</t>
-  </si>
-  <si>
     <t>Tanggal Kontrak</t>
   </si>
   <si>
     <t>Nomor Kontrak</t>
+  </si>
+  <si>
+    <t>Rekap Kontrak Pengadaan</t>
   </si>
 </sst>
 </file>
@@ -455,7 +455,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -493,10 +493,10 @@
         <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>1</v>

</xml_diff>